<commit_message>
Sync from ryanbr/noop 971d0d9f
</commit_message>
<xml_diff>
--- a/docs/lift-log-program-template.xlsx
+++ b/docs/lift-log-program-template.xlsx
@@ -73,8 +73,9 @@
     <col min="6" max="6" width="7" customWidth="1"/>
     <col min="7" max="7" width="7" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="34" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -120,10 +121,15 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Target max RPE</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rest sec</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Note</t>
         </is>
@@ -140,6 +146,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" s="2"/>
@@ -152,6 +159,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" s="2"/>
@@ -164,6 +172,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" s="2"/>
@@ -176,6 +185,7 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" s="2"/>
@@ -188,6 +198,7 @@
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" s="2"/>
@@ -200,6 +211,7 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" s="2"/>
@@ -212,6 +224,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" s="2"/>
@@ -224,6 +237,7 @@
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" s="2"/>
@@ -236,6 +250,7 @@
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" s="2"/>
@@ -248,6 +263,7 @@
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" s="2"/>
@@ -260,6 +276,7 @@
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" s="2"/>
@@ -272,6 +289,7 @@
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" s="2"/>
@@ -284,6 +302,7 @@
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" s="2"/>
@@ -296,6 +315,7 @@
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" s="2"/>
@@ -308,6 +328,7 @@
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" s="2"/>
@@ -320,6 +341,7 @@
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" s="2"/>
@@ -332,6 +354,7 @@
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" s="2"/>
@@ -344,6 +367,7 @@
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" s="2"/>
@@ -356,6 +380,7 @@
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" s="2"/>
@@ -368,6 +393,7 @@
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
     </row>
     <row r="22">
       <c r="A22" s="2"/>
@@ -380,6 +406,7 @@
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
     </row>
     <row r="23">
       <c r="A23" s="2"/>
@@ -392,6 +419,7 @@
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
     </row>
     <row r="24">
       <c r="A24" s="2"/>
@@ -404,6 +432,7 @@
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
     </row>
     <row r="25">
       <c r="A25" s="2"/>
@@ -416,6 +445,7 @@
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
     </row>
     <row r="26">
       <c r="A26" s="2"/>
@@ -428,6 +458,7 @@
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
     </row>
     <row r="27">
       <c r="A27" s="2"/>
@@ -440,6 +471,7 @@
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
     </row>
     <row r="28">
       <c r="A28" s="2"/>
@@ -452,6 +484,7 @@
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
     </row>
     <row r="29">
       <c r="A29" s="2"/>
@@ -464,6 +497,7 @@
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
     </row>
     <row r="30">
       <c r="A30" s="2"/>
@@ -476,6 +510,7 @@
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
     </row>
     <row r="31">
       <c r="A31" s="2"/>
@@ -488,6 +523,7 @@
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
     </row>
     <row r="32">
       <c r="A32" s="2"/>
@@ -500,6 +536,7 @@
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
     </row>
     <row r="33">
       <c r="A33" s="2"/>
@@ -512,6 +549,7 @@
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
     </row>
     <row r="34">
       <c r="A34" s="2"/>
@@ -524,6 +562,7 @@
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
     </row>
     <row r="35">
       <c r="A35" s="2"/>
@@ -536,6 +575,7 @@
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
     </row>
     <row r="36">
       <c r="A36" s="2"/>
@@ -548,6 +588,7 @@
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
     </row>
     <row r="37">
       <c r="A37" s="2"/>
@@ -560,6 +601,7 @@
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
     </row>
     <row r="38">
       <c r="A38" s="2"/>
@@ -572,6 +614,7 @@
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
     </row>
     <row r="39">
       <c r="A39" s="2"/>
@@ -584,6 +627,7 @@
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
     </row>
     <row r="40">
       <c r="A40" s="2"/>
@@ -596,6 +640,7 @@
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
     </row>
     <row r="41">
       <c r="A41" s="2"/>
@@ -608,6 +653,7 @@
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
     </row>
     <row r="42">
       <c r="A42" s="2"/>
@@ -620,6 +666,7 @@
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
     </row>
     <row r="43">
       <c r="A43" s="2"/>
@@ -632,6 +679,7 @@
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
     </row>
     <row r="44">
       <c r="A44" s="2"/>
@@ -644,6 +692,7 @@
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
     </row>
     <row r="45">
       <c r="A45" s="2"/>
@@ -656,6 +705,7 @@
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
     </row>
     <row r="46">
       <c r="A46" s="2"/>
@@ -668,6 +718,7 @@
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
     </row>
     <row r="47">
       <c r="A47" s="2"/>
@@ -680,6 +731,7 @@
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
     </row>
     <row r="48">
       <c r="A48" s="2"/>
@@ -692,6 +744,7 @@
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
     </row>
     <row r="49">
       <c r="A49" s="2"/>
@@ -704,6 +757,7 @@
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
+      <c r="K49" s="2"/>
     </row>
     <row r="50">
       <c r="A50" s="2"/>
@@ -716,6 +770,7 @@
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
+      <c r="K50" s="2"/>
     </row>
     <row r="51">
       <c r="A51" s="2"/>
@@ -728,6 +783,7 @@
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
     </row>
     <row r="52">
       <c r="A52" s="2"/>
@@ -740,6 +796,7 @@
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
     </row>
     <row r="53">
       <c r="A53" s="2"/>
@@ -752,6 +809,7 @@
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
     </row>
     <row r="54">
       <c r="A54" s="2"/>
@@ -764,6 +822,7 @@
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
+      <c r="K54" s="2"/>
     </row>
     <row r="55">
       <c r="A55" s="2"/>
@@ -776,6 +835,7 @@
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
+      <c r="K55" s="2"/>
     </row>
     <row r="56">
       <c r="A56" s="2"/>
@@ -788,6 +848,7 @@
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
+      <c r="K56" s="2"/>
     </row>
     <row r="57">
       <c r="A57" s="2"/>
@@ -800,6 +861,7 @@
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
+      <c r="K57" s="2"/>
     </row>
     <row r="58">
       <c r="A58" s="2"/>
@@ -812,6 +874,7 @@
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
+      <c r="K58" s="2"/>
     </row>
     <row r="59">
       <c r="A59" s="2"/>
@@ -824,6 +887,7 @@
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
     </row>
     <row r="60">
       <c r="A60" s="2"/>
@@ -836,6 +900,7 @@
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
+      <c r="K60" s="2"/>
     </row>
     <row r="61">
       <c r="A61" s="2"/>
@@ -848,6 +913,7 @@
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
     </row>
     <row r="62">
       <c r="A62" s="2"/>
@@ -860,6 +926,7 @@
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
+      <c r="K62" s="2"/>
     </row>
     <row r="63">
       <c r="A63" s="2"/>
@@ -872,6 +939,7 @@
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
+      <c r="K63" s="2"/>
     </row>
     <row r="64">
       <c r="A64" s="2"/>
@@ -884,6 +952,7 @@
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
+      <c r="K64" s="2"/>
     </row>
     <row r="65">
       <c r="A65" s="2"/>
@@ -896,6 +965,7 @@
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
+      <c r="K65" s="2"/>
     </row>
     <row r="66">
       <c r="A66" s="2"/>
@@ -908,6 +978,7 @@
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
     </row>
     <row r="67">
       <c r="A67" s="2"/>
@@ -920,6 +991,7 @@
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
+      <c r="K67" s="2"/>
     </row>
     <row r="68">
       <c r="A68" s="2"/>
@@ -932,6 +1004,7 @@
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
+      <c r="K68" s="2"/>
     </row>
     <row r="69">
       <c r="A69" s="2"/>
@@ -944,6 +1017,7 @@
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
+      <c r="K69" s="2"/>
     </row>
     <row r="70">
       <c r="A70" s="2"/>
@@ -956,6 +1030,7 @@
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
+      <c r="K70" s="2"/>
     </row>
     <row r="71">
       <c r="A71" s="2"/>
@@ -968,6 +1043,7 @@
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
+      <c r="K71" s="2"/>
     </row>
     <row r="72">
       <c r="A72" s="2"/>
@@ -980,6 +1056,7 @@
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
+      <c r="K72" s="2"/>
     </row>
     <row r="73">
       <c r="A73" s="2"/>
@@ -992,6 +1069,7 @@
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
+      <c r="K73" s="2"/>
     </row>
     <row r="74">
       <c r="A74" s="2"/>
@@ -1004,6 +1082,7 @@
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
+      <c r="K74" s="2"/>
     </row>
     <row r="75">
       <c r="A75" s="2"/>
@@ -1016,6 +1095,7 @@
       <c r="H75" s="2"/>
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
+      <c r="K75" s="2"/>
     </row>
     <row r="76">
       <c r="A76" s="2"/>
@@ -1028,6 +1108,7 @@
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
+      <c r="K76" s="2"/>
     </row>
     <row r="77">
       <c r="A77" s="2"/>
@@ -1040,6 +1121,7 @@
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
+      <c r="K77" s="2"/>
     </row>
     <row r="78">
       <c r="A78" s="2"/>
@@ -1052,6 +1134,7 @@
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
+      <c r="K78" s="2"/>
     </row>
     <row r="79">
       <c r="A79" s="2"/>
@@ -1064,6 +1147,7 @@
       <c r="H79" s="2"/>
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
+      <c r="K79" s="2"/>
     </row>
     <row r="80">
       <c r="A80" s="2"/>
@@ -1076,6 +1160,7 @@
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
+      <c r="K80" s="2"/>
     </row>
     <row r="81">
       <c r="A81" s="2"/>
@@ -1088,6 +1173,7 @@
       <c r="H81" s="2"/>
       <c r="I81" s="2"/>
       <c r="J81" s="2"/>
+      <c r="K81" s="2"/>
     </row>
     <row r="82">
       <c r="A82" s="2"/>
@@ -1100,6 +1186,7 @@
       <c r="H82" s="2"/>
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
+      <c r="K82" s="2"/>
     </row>
     <row r="83">
       <c r="A83" s="2"/>
@@ -1112,6 +1199,7 @@
       <c r="H83" s="2"/>
       <c r="I83" s="2"/>
       <c r="J83" s="2"/>
+      <c r="K83" s="2"/>
     </row>
     <row r="84">
       <c r="A84" s="2"/>
@@ -1124,6 +1212,7 @@
       <c r="H84" s="2"/>
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
+      <c r="K84" s="2"/>
     </row>
     <row r="85">
       <c r="A85" s="2"/>
@@ -1136,6 +1225,7 @@
       <c r="H85" s="2"/>
       <c r="I85" s="2"/>
       <c r="J85" s="2"/>
+      <c r="K85" s="2"/>
     </row>
     <row r="86">
       <c r="A86" s="2"/>
@@ -1148,6 +1238,7 @@
       <c r="H86" s="2"/>
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
+      <c r="K86" s="2"/>
     </row>
     <row r="87">
       <c r="A87" s="2"/>
@@ -1160,6 +1251,7 @@
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
+      <c r="K87" s="2"/>
     </row>
     <row r="88">
       <c r="A88" s="2"/>
@@ -1172,6 +1264,7 @@
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
+      <c r="K88" s="2"/>
     </row>
     <row r="89">
       <c r="A89" s="2"/>
@@ -1184,6 +1277,7 @@
       <c r="H89" s="2"/>
       <c r="I89" s="2"/>
       <c r="J89" s="2"/>
+      <c r="K89" s="2"/>
     </row>
     <row r="90">
       <c r="A90" s="2"/>
@@ -1196,6 +1290,7 @@
       <c r="H90" s="2"/>
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
+      <c r="K90" s="2"/>
     </row>
     <row r="91">
       <c r="A91" s="2"/>
@@ -1208,6 +1303,7 @@
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
+      <c r="K91" s="2"/>
     </row>
     <row r="92">
       <c r="A92" s="2"/>
@@ -1220,6 +1316,7 @@
       <c r="H92" s="2"/>
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
+      <c r="K92" s="2"/>
     </row>
     <row r="93">
       <c r="A93" s="2"/>
@@ -1232,6 +1329,7 @@
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
+      <c r="K93" s="2"/>
     </row>
     <row r="94">
       <c r="A94" s="2"/>
@@ -1244,6 +1342,7 @@
       <c r="H94" s="2"/>
       <c r="I94" s="2"/>
       <c r="J94" s="2"/>
+      <c r="K94" s="2"/>
     </row>
     <row r="95">
       <c r="A95" s="2"/>
@@ -1256,6 +1355,7 @@
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
+      <c r="K95" s="2"/>
     </row>
     <row r="96">
       <c r="A96" s="2"/>
@@ -1268,6 +1368,7 @@
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
+      <c r="K96" s="2"/>
     </row>
     <row r="97">
       <c r="A97" s="2"/>
@@ -1280,6 +1381,7 @@
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
+      <c r="K97" s="2"/>
     </row>
     <row r="98">
       <c r="A98" s="2"/>
@@ -1292,6 +1394,7 @@
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
       <c r="J98" s="2"/>
+      <c r="K98" s="2"/>
     </row>
     <row r="99">
       <c r="A99" s="2"/>
@@ -1304,6 +1407,7 @@
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
       <c r="J99" s="2"/>
+      <c r="K99" s="2"/>
     </row>
     <row r="100">
       <c r="A100" s="2"/>
@@ -1316,6 +1420,7 @@
       <c r="H100" s="2"/>
       <c r="I100" s="2"/>
       <c r="J100" s="2"/>
+      <c r="K100" s="2"/>
     </row>
     <row r="101">
       <c r="A101" s="2"/>
@@ -1328,6 +1433,7 @@
       <c r="H101" s="2"/>
       <c r="I101" s="2"/>
       <c r="J101" s="2"/>
+      <c r="K101" s="2"/>
     </row>
     <row r="102">
       <c r="A102" s="2"/>
@@ -1340,6 +1446,7 @@
       <c r="H102" s="2"/>
       <c r="I102" s="2"/>
       <c r="J102" s="2"/>
+      <c r="K102" s="2"/>
     </row>
     <row r="103">
       <c r="A103" s="2"/>
@@ -1352,6 +1459,7 @@
       <c r="H103" s="2"/>
       <c r="I103" s="2"/>
       <c r="J103" s="2"/>
+      <c r="K103" s="2"/>
     </row>
     <row r="104">
       <c r="A104" s="2"/>
@@ -1364,6 +1472,7 @@
       <c r="H104" s="2"/>
       <c r="I104" s="2"/>
       <c r="J104" s="2"/>
+      <c r="K104" s="2"/>
     </row>
     <row r="105">
       <c r="A105" s="2"/>
@@ -1376,6 +1485,7 @@
       <c r="H105" s="2"/>
       <c r="I105" s="2"/>
       <c r="J105" s="2"/>
+      <c r="K105" s="2"/>
     </row>
     <row r="106">
       <c r="A106" s="2"/>
@@ -1388,6 +1498,7 @@
       <c r="H106" s="2"/>
       <c r="I106" s="2"/>
       <c r="J106" s="2"/>
+      <c r="K106" s="2"/>
     </row>
     <row r="107">
       <c r="A107" s="2"/>
@@ -1400,6 +1511,7 @@
       <c r="H107" s="2"/>
       <c r="I107" s="2"/>
       <c r="J107" s="2"/>
+      <c r="K107" s="2"/>
     </row>
     <row r="108">
       <c r="A108" s="2"/>
@@ -1412,6 +1524,7 @@
       <c r="H108" s="2"/>
       <c r="I108" s="2"/>
       <c r="J108" s="2"/>
+      <c r="K108" s="2"/>
     </row>
     <row r="109">
       <c r="A109" s="2"/>
@@ -1424,6 +1537,7 @@
       <c r="H109" s="2"/>
       <c r="I109" s="2"/>
       <c r="J109" s="2"/>
+      <c r="K109" s="2"/>
     </row>
     <row r="110">
       <c r="A110" s="2"/>
@@ -1436,6 +1550,7 @@
       <c r="H110" s="2"/>
       <c r="I110" s="2"/>
       <c r="J110" s="2"/>
+      <c r="K110" s="2"/>
     </row>
     <row r="111">
       <c r="A111" s="2"/>
@@ -1448,6 +1563,7 @@
       <c r="H111" s="2"/>
       <c r="I111" s="2"/>
       <c r="J111" s="2"/>
+      <c r="K111" s="2"/>
     </row>
     <row r="112">
       <c r="A112" s="2"/>
@@ -1460,6 +1576,7 @@
       <c r="H112" s="2"/>
       <c r="I112" s="2"/>
       <c r="J112" s="2"/>
+      <c r="K112" s="2"/>
     </row>
     <row r="113">
       <c r="A113" s="2"/>
@@ -1472,6 +1589,7 @@
       <c r="H113" s="2"/>
       <c r="I113" s="2"/>
       <c r="J113" s="2"/>
+      <c r="K113" s="2"/>
     </row>
     <row r="114">
       <c r="A114" s="2"/>
@@ -1484,6 +1602,7 @@
       <c r="H114" s="2"/>
       <c r="I114" s="2"/>
       <c r="J114" s="2"/>
+      <c r="K114" s="2"/>
     </row>
     <row r="115">
       <c r="A115" s="2"/>
@@ -1496,6 +1615,7 @@
       <c r="H115" s="2"/>
       <c r="I115" s="2"/>
       <c r="J115" s="2"/>
+      <c r="K115" s="2"/>
     </row>
     <row r="116">
       <c r="A116" s="2"/>
@@ -1508,6 +1628,7 @@
       <c r="H116" s="2"/>
       <c r="I116" s="2"/>
       <c r="J116" s="2"/>
+      <c r="K116" s="2"/>
     </row>
     <row r="117">
       <c r="A117" s="2"/>
@@ -1520,6 +1641,7 @@
       <c r="H117" s="2"/>
       <c r="I117" s="2"/>
       <c r="J117" s="2"/>
+      <c r="K117" s="2"/>
     </row>
     <row r="118">
       <c r="A118" s="2"/>
@@ -1532,6 +1654,7 @@
       <c r="H118" s="2"/>
       <c r="I118" s="2"/>
       <c r="J118" s="2"/>
+      <c r="K118" s="2"/>
     </row>
     <row r="119">
       <c r="A119" s="2"/>
@@ -1544,6 +1667,7 @@
       <c r="H119" s="2"/>
       <c r="I119" s="2"/>
       <c r="J119" s="2"/>
+      <c r="K119" s="2"/>
     </row>
     <row r="120">
       <c r="A120" s="2"/>
@@ -1556,6 +1680,7 @@
       <c r="H120" s="2"/>
       <c r="I120" s="2"/>
       <c r="J120" s="2"/>
+      <c r="K120" s="2"/>
     </row>
     <row r="121">
       <c r="A121" s="2"/>
@@ -1568,6 +1693,7 @@
       <c r="H121" s="2"/>
       <c r="I121" s="2"/>
       <c r="J121" s="2"/>
+      <c r="K121" s="2"/>
     </row>
     <row r="122">
       <c r="A122" s="2"/>
@@ -1580,6 +1706,7 @@
       <c r="H122" s="2"/>
       <c r="I122" s="2"/>
       <c r="J122" s="2"/>
+      <c r="K122" s="2"/>
     </row>
     <row r="123">
       <c r="A123" s="2"/>
@@ -1592,6 +1719,7 @@
       <c r="H123" s="2"/>
       <c r="I123" s="2"/>
       <c r="J123" s="2"/>
+      <c r="K123" s="2"/>
     </row>
     <row r="124">
       <c r="A124" s="2"/>
@@ -1604,6 +1732,7 @@
       <c r="H124" s="2"/>
       <c r="I124" s="2"/>
       <c r="J124" s="2"/>
+      <c r="K124" s="2"/>
     </row>
     <row r="125">
       <c r="A125" s="2"/>
@@ -1616,6 +1745,7 @@
       <c r="H125" s="2"/>
       <c r="I125" s="2"/>
       <c r="J125" s="2"/>
+      <c r="K125" s="2"/>
     </row>
     <row r="126">
       <c r="A126" s="2"/>
@@ -1628,6 +1758,7 @@
       <c r="H126" s="2"/>
       <c r="I126" s="2"/>
       <c r="J126" s="2"/>
+      <c r="K126" s="2"/>
     </row>
     <row r="127">
       <c r="A127" s="2"/>
@@ -1640,6 +1771,7 @@
       <c r="H127" s="2"/>
       <c r="I127" s="2"/>
       <c r="J127" s="2"/>
+      <c r="K127" s="2"/>
     </row>
     <row r="128">
       <c r="A128" s="2"/>
@@ -1652,6 +1784,7 @@
       <c r="H128" s="2"/>
       <c r="I128" s="2"/>
       <c r="J128" s="2"/>
+      <c r="K128" s="2"/>
     </row>
     <row r="129">
       <c r="A129" s="2"/>
@@ -1664,6 +1797,7 @@
       <c r="H129" s="2"/>
       <c r="I129" s="2"/>
       <c r="J129" s="2"/>
+      <c r="K129" s="2"/>
     </row>
     <row r="130">
       <c r="A130" s="2"/>
@@ -1676,6 +1810,7 @@
       <c r="H130" s="2"/>
       <c r="I130" s="2"/>
       <c r="J130" s="2"/>
+      <c r="K130" s="2"/>
     </row>
     <row r="131">
       <c r="A131" s="2"/>
@@ -1688,6 +1823,7 @@
       <c r="H131" s="2"/>
       <c r="I131" s="2"/>
       <c r="J131" s="2"/>
+      <c r="K131" s="2"/>
     </row>
     <row r="132">
       <c r="A132" s="2"/>
@@ -1700,6 +1836,7 @@
       <c r="H132" s="2"/>
       <c r="I132" s="2"/>
       <c r="J132" s="2"/>
+      <c r="K132" s="2"/>
     </row>
     <row r="133">
       <c r="A133" s="2"/>
@@ -1712,6 +1849,7 @@
       <c r="H133" s="2"/>
       <c r="I133" s="2"/>
       <c r="J133" s="2"/>
+      <c r="K133" s="2"/>
     </row>
     <row r="134">
       <c r="A134" s="2"/>
@@ -1724,6 +1862,7 @@
       <c r="H134" s="2"/>
       <c r="I134" s="2"/>
       <c r="J134" s="2"/>
+      <c r="K134" s="2"/>
     </row>
     <row r="135">
       <c r="A135" s="2"/>
@@ -1736,6 +1875,7 @@
       <c r="H135" s="2"/>
       <c r="I135" s="2"/>
       <c r="J135" s="2"/>
+      <c r="K135" s="2"/>
     </row>
     <row r="136">
       <c r="A136" s="2"/>
@@ -1748,6 +1888,7 @@
       <c r="H136" s="2"/>
       <c r="I136" s="2"/>
       <c r="J136" s="2"/>
+      <c r="K136" s="2"/>
     </row>
     <row r="137">
       <c r="A137" s="2"/>
@@ -1760,6 +1901,7 @@
       <c r="H137" s="2"/>
       <c r="I137" s="2"/>
       <c r="J137" s="2"/>
+      <c r="K137" s="2"/>
     </row>
     <row r="138">
       <c r="A138" s="2"/>
@@ -1772,6 +1914,7 @@
       <c r="H138" s="2"/>
       <c r="I138" s="2"/>
       <c r="J138" s="2"/>
+      <c r="K138" s="2"/>
     </row>
     <row r="139">
       <c r="A139" s="2"/>
@@ -1784,6 +1927,7 @@
       <c r="H139" s="2"/>
       <c r="I139" s="2"/>
       <c r="J139" s="2"/>
+      <c r="K139" s="2"/>
     </row>
     <row r="140">
       <c r="A140" s="2"/>
@@ -1796,6 +1940,7 @@
       <c r="H140" s="2"/>
       <c r="I140" s="2"/>
       <c r="J140" s="2"/>
+      <c r="K140" s="2"/>
     </row>
     <row r="141">
       <c r="A141" s="2"/>
@@ -1808,6 +1953,7 @@
       <c r="H141" s="2"/>
       <c r="I141" s="2"/>
       <c r="J141" s="2"/>
+      <c r="K141" s="2"/>
     </row>
     <row r="142">
       <c r="A142" s="2"/>
@@ -1820,6 +1966,7 @@
       <c r="H142" s="2"/>
       <c r="I142" s="2"/>
       <c r="J142" s="2"/>
+      <c r="K142" s="2"/>
     </row>
     <row r="143">
       <c r="A143" s="2"/>
@@ -1832,6 +1979,7 @@
       <c r="H143" s="2"/>
       <c r="I143" s="2"/>
       <c r="J143" s="2"/>
+      <c r="K143" s="2"/>
     </row>
     <row r="144">
       <c r="A144" s="2"/>
@@ -1844,6 +1992,7 @@
       <c r="H144" s="2"/>
       <c r="I144" s="2"/>
       <c r="J144" s="2"/>
+      <c r="K144" s="2"/>
     </row>
     <row r="145">
       <c r="A145" s="2"/>
@@ -1856,6 +2005,7 @@
       <c r="H145" s="2"/>
       <c r="I145" s="2"/>
       <c r="J145" s="2"/>
+      <c r="K145" s="2"/>
     </row>
     <row r="146">
       <c r="A146" s="2"/>
@@ -1868,6 +2018,7 @@
       <c r="H146" s="2"/>
       <c r="I146" s="2"/>
       <c r="J146" s="2"/>
+      <c r="K146" s="2"/>
     </row>
     <row r="147">
       <c r="A147" s="2"/>
@@ -1880,6 +2031,7 @@
       <c r="H147" s="2"/>
       <c r="I147" s="2"/>
       <c r="J147" s="2"/>
+      <c r="K147" s="2"/>
     </row>
     <row r="148">
       <c r="A148" s="2"/>
@@ -1892,6 +2044,7 @@
       <c r="H148" s="2"/>
       <c r="I148" s="2"/>
       <c r="J148" s="2"/>
+      <c r="K148" s="2"/>
     </row>
     <row r="149">
       <c r="A149" s="2"/>
@@ -1904,6 +2057,7 @@
       <c r="H149" s="2"/>
       <c r="I149" s="2"/>
       <c r="J149" s="2"/>
+      <c r="K149" s="2"/>
     </row>
     <row r="150">
       <c r="A150" s="2"/>
@@ -1916,6 +2070,7 @@
       <c r="H150" s="2"/>
       <c r="I150" s="2"/>
       <c r="J150" s="2"/>
+      <c r="K150" s="2"/>
     </row>
     <row r="151">
       <c r="A151" s="2"/>
@@ -1928,6 +2083,7 @@
       <c r="H151" s="2"/>
       <c r="I151" s="2"/>
       <c r="J151" s="2"/>
+      <c r="K151" s="2"/>
     </row>
     <row r="152">
       <c r="A152" s="2"/>
@@ -1940,6 +2096,7 @@
       <c r="H152" s="2"/>
       <c r="I152" s="2"/>
       <c r="J152" s="2"/>
+      <c r="K152" s="2"/>
     </row>
     <row r="153">
       <c r="A153" s="2"/>
@@ -1952,6 +2109,7 @@
       <c r="H153" s="2"/>
       <c r="I153" s="2"/>
       <c r="J153" s="2"/>
+      <c r="K153" s="2"/>
     </row>
     <row r="154">
       <c r="A154" s="2"/>
@@ -1964,6 +2122,7 @@
       <c r="H154" s="2"/>
       <c r="I154" s="2"/>
       <c r="J154" s="2"/>
+      <c r="K154" s="2"/>
     </row>
     <row r="155">
       <c r="A155" s="2"/>
@@ -1976,6 +2135,7 @@
       <c r="H155" s="2"/>
       <c r="I155" s="2"/>
       <c r="J155" s="2"/>
+      <c r="K155" s="2"/>
     </row>
     <row r="156">
       <c r="A156" s="2"/>
@@ -1988,6 +2148,7 @@
       <c r="H156" s="2"/>
       <c r="I156" s="2"/>
       <c r="J156" s="2"/>
+      <c r="K156" s="2"/>
     </row>
     <row r="157">
       <c r="A157" s="2"/>
@@ -2000,6 +2161,7 @@
       <c r="H157" s="2"/>
       <c r="I157" s="2"/>
       <c r="J157" s="2"/>
+      <c r="K157" s="2"/>
     </row>
     <row r="158">
       <c r="A158" s="2"/>
@@ -2012,6 +2174,7 @@
       <c r="H158" s="2"/>
       <c r="I158" s="2"/>
       <c r="J158" s="2"/>
+      <c r="K158" s="2"/>
     </row>
     <row r="159">
       <c r="A159" s="2"/>
@@ -2024,6 +2187,7 @@
       <c r="H159" s="2"/>
       <c r="I159" s="2"/>
       <c r="J159" s="2"/>
+      <c r="K159" s="2"/>
     </row>
     <row r="160">
       <c r="A160" s="2"/>
@@ -2036,6 +2200,7 @@
       <c r="H160" s="2"/>
       <c r="I160" s="2"/>
       <c r="J160" s="2"/>
+      <c r="K160" s="2"/>
     </row>
     <row r="161">
       <c r="A161" s="2"/>
@@ -2048,6 +2213,7 @@
       <c r="H161" s="2"/>
       <c r="I161" s="2"/>
       <c r="J161" s="2"/>
+      <c r="K161" s="2"/>
     </row>
     <row r="162">
       <c r="A162" s="2"/>
@@ -2060,6 +2226,7 @@
       <c r="H162" s="2"/>
       <c r="I162" s="2"/>
       <c r="J162" s="2"/>
+      <c r="K162" s="2"/>
     </row>
     <row r="163">
       <c r="A163" s="2"/>
@@ -2072,6 +2239,7 @@
       <c r="H163" s="2"/>
       <c r="I163" s="2"/>
       <c r="J163" s="2"/>
+      <c r="K163" s="2"/>
     </row>
     <row r="164">
       <c r="A164" s="2"/>
@@ -2084,6 +2252,7 @@
       <c r="H164" s="2"/>
       <c r="I164" s="2"/>
       <c r="J164" s="2"/>
+      <c r="K164" s="2"/>
     </row>
     <row r="165">
       <c r="A165" s="2"/>
@@ -2096,6 +2265,7 @@
       <c r="H165" s="2"/>
       <c r="I165" s="2"/>
       <c r="J165" s="2"/>
+      <c r="K165" s="2"/>
     </row>
     <row r="166">
       <c r="A166" s="2"/>
@@ -2108,6 +2278,7 @@
       <c r="H166" s="2"/>
       <c r="I166" s="2"/>
       <c r="J166" s="2"/>
+      <c r="K166" s="2"/>
     </row>
     <row r="167">
       <c r="A167" s="2"/>
@@ -2120,6 +2291,7 @@
       <c r="H167" s="2"/>
       <c r="I167" s="2"/>
       <c r="J167" s="2"/>
+      <c r="K167" s="2"/>
     </row>
     <row r="168">
       <c r="A168" s="2"/>
@@ -2132,6 +2304,7 @@
       <c r="H168" s="2"/>
       <c r="I168" s="2"/>
       <c r="J168" s="2"/>
+      <c r="K168" s="2"/>
     </row>
     <row r="169">
       <c r="A169" s="2"/>
@@ -2144,6 +2317,7 @@
       <c r="H169" s="2"/>
       <c r="I169" s="2"/>
       <c r="J169" s="2"/>
+      <c r="K169" s="2"/>
     </row>
     <row r="170">
       <c r="A170" s="2"/>
@@ -2156,6 +2330,7 @@
       <c r="H170" s="2"/>
       <c r="I170" s="2"/>
       <c r="J170" s="2"/>
+      <c r="K170" s="2"/>
     </row>
     <row r="171">
       <c r="A171" s="2"/>
@@ -2168,6 +2343,7 @@
       <c r="H171" s="2"/>
       <c r="I171" s="2"/>
       <c r="J171" s="2"/>
+      <c r="K171" s="2"/>
     </row>
     <row r="172">
       <c r="A172" s="2"/>
@@ -2180,6 +2356,7 @@
       <c r="H172" s="2"/>
       <c r="I172" s="2"/>
       <c r="J172" s="2"/>
+      <c r="K172" s="2"/>
     </row>
     <row r="173">
       <c r="A173" s="2"/>
@@ -2192,6 +2369,7 @@
       <c r="H173" s="2"/>
       <c r="I173" s="2"/>
       <c r="J173" s="2"/>
+      <c r="K173" s="2"/>
     </row>
     <row r="174">
       <c r="A174" s="2"/>
@@ -2204,6 +2382,7 @@
       <c r="H174" s="2"/>
       <c r="I174" s="2"/>
       <c r="J174" s="2"/>
+      <c r="K174" s="2"/>
     </row>
     <row r="175">
       <c r="A175" s="2"/>
@@ -2216,6 +2395,7 @@
       <c r="H175" s="2"/>
       <c r="I175" s="2"/>
       <c r="J175" s="2"/>
+      <c r="K175" s="2"/>
     </row>
     <row r="176">
       <c r="A176" s="2"/>
@@ -2228,6 +2408,7 @@
       <c r="H176" s="2"/>
       <c r="I176" s="2"/>
       <c r="J176" s="2"/>
+      <c r="K176" s="2"/>
     </row>
     <row r="177">
       <c r="A177" s="2"/>
@@ -2240,6 +2421,7 @@
       <c r="H177" s="2"/>
       <c r="I177" s="2"/>
       <c r="J177" s="2"/>
+      <c r="K177" s="2"/>
     </row>
     <row r="178">
       <c r="A178" s="2"/>
@@ -2252,6 +2434,7 @@
       <c r="H178" s="2"/>
       <c r="I178" s="2"/>
       <c r="J178" s="2"/>
+      <c r="K178" s="2"/>
     </row>
     <row r="179">
       <c r="A179" s="2"/>
@@ -2264,6 +2447,7 @@
       <c r="H179" s="2"/>
       <c r="I179" s="2"/>
       <c r="J179" s="2"/>
+      <c r="K179" s="2"/>
     </row>
     <row r="180">
       <c r="A180" s="2"/>
@@ -2276,6 +2460,7 @@
       <c r="H180" s="2"/>
       <c r="I180" s="2"/>
       <c r="J180" s="2"/>
+      <c r="K180" s="2"/>
     </row>
     <row r="181">
       <c r="A181" s="2"/>
@@ -2288,6 +2473,7 @@
       <c r="H181" s="2"/>
       <c r="I181" s="2"/>
       <c r="J181" s="2"/>
+      <c r="K181" s="2"/>
     </row>
     <row r="182">
       <c r="A182" s="2"/>
@@ -2300,6 +2486,7 @@
       <c r="H182" s="2"/>
       <c r="I182" s="2"/>
       <c r="J182" s="2"/>
+      <c r="K182" s="2"/>
     </row>
     <row r="183">
       <c r="A183" s="2"/>
@@ -2312,6 +2499,7 @@
       <c r="H183" s="2"/>
       <c r="I183" s="2"/>
       <c r="J183" s="2"/>
+      <c r="K183" s="2"/>
     </row>
     <row r="184">
       <c r="A184" s="2"/>
@@ -2324,6 +2512,7 @@
       <c r="H184" s="2"/>
       <c r="I184" s="2"/>
       <c r="J184" s="2"/>
+      <c r="K184" s="2"/>
     </row>
     <row r="185">
       <c r="A185" s="2"/>
@@ -2336,6 +2525,7 @@
       <c r="H185" s="2"/>
       <c r="I185" s="2"/>
       <c r="J185" s="2"/>
+      <c r="K185" s="2"/>
     </row>
     <row r="186">
       <c r="A186" s="2"/>
@@ -2348,6 +2538,7 @@
       <c r="H186" s="2"/>
       <c r="I186" s="2"/>
       <c r="J186" s="2"/>
+      <c r="K186" s="2"/>
     </row>
     <row r="187">
       <c r="A187" s="2"/>
@@ -2360,6 +2551,7 @@
       <c r="H187" s="2"/>
       <c r="I187" s="2"/>
       <c r="J187" s="2"/>
+      <c r="K187" s="2"/>
     </row>
     <row r="188">
       <c r="A188" s="2"/>
@@ -2372,6 +2564,7 @@
       <c r="H188" s="2"/>
       <c r="I188" s="2"/>
       <c r="J188" s="2"/>
+      <c r="K188" s="2"/>
     </row>
     <row r="189">
       <c r="A189" s="2"/>
@@ -2384,6 +2577,7 @@
       <c r="H189" s="2"/>
       <c r="I189" s="2"/>
       <c r="J189" s="2"/>
+      <c r="K189" s="2"/>
     </row>
     <row r="190">
       <c r="A190" s="2"/>
@@ -2396,6 +2590,7 @@
       <c r="H190" s="2"/>
       <c r="I190" s="2"/>
       <c r="J190" s="2"/>
+      <c r="K190" s="2"/>
     </row>
     <row r="191">
       <c r="A191" s="2"/>
@@ -2408,6 +2603,7 @@
       <c r="H191" s="2"/>
       <c r="I191" s="2"/>
       <c r="J191" s="2"/>
+      <c r="K191" s="2"/>
     </row>
     <row r="192">
       <c r="A192" s="2"/>
@@ -2420,6 +2616,7 @@
       <c r="H192" s="2"/>
       <c r="I192" s="2"/>
       <c r="J192" s="2"/>
+      <c r="K192" s="2"/>
     </row>
     <row r="193">
       <c r="A193" s="2"/>
@@ -2432,6 +2629,7 @@
       <c r="H193" s="2"/>
       <c r="I193" s="2"/>
       <c r="J193" s="2"/>
+      <c r="K193" s="2"/>
     </row>
     <row r="194">
       <c r="A194" s="2"/>
@@ -2444,6 +2642,7 @@
       <c r="H194" s="2"/>
       <c r="I194" s="2"/>
       <c r="J194" s="2"/>
+      <c r="K194" s="2"/>
     </row>
     <row r="195">
       <c r="A195" s="2"/>
@@ -2456,6 +2655,7 @@
       <c r="H195" s="2"/>
       <c r="I195" s="2"/>
       <c r="J195" s="2"/>
+      <c r="K195" s="2"/>
     </row>
     <row r="196">
       <c r="A196" s="2"/>
@@ -2468,6 +2668,7 @@
       <c r="H196" s="2"/>
       <c r="I196" s="2"/>
       <c r="J196" s="2"/>
+      <c r="K196" s="2"/>
     </row>
     <row r="197">
       <c r="A197" s="2"/>
@@ -2480,6 +2681,7 @@
       <c r="H197" s="2"/>
       <c r="I197" s="2"/>
       <c r="J197" s="2"/>
+      <c r="K197" s="2"/>
     </row>
     <row r="198">
       <c r="A198" s="2"/>
@@ -2492,6 +2694,7 @@
       <c r="H198" s="2"/>
       <c r="I198" s="2"/>
       <c r="J198" s="2"/>
+      <c r="K198" s="2"/>
     </row>
     <row r="199">
       <c r="A199" s="2"/>
@@ -2504,6 +2707,7 @@
       <c r="H199" s="2"/>
       <c r="I199" s="2"/>
       <c r="J199" s="2"/>
+      <c r="K199" s="2"/>
     </row>
     <row r="200">
       <c r="A200" s="2"/>
@@ -2516,6 +2720,7 @@
       <c r="H200" s="2"/>
       <c r="I200" s="2"/>
       <c r="J200" s="2"/>
+      <c r="K200" s="2"/>
     </row>
     <row r="201">
       <c r="A201" s="2"/>
@@ -2528,15 +2733,20 @@
       <c r="H201" s="2"/>
       <c r="I201" s="2"/>
       <c r="J201" s="2"/>
+      <c r="K201" s="2"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="0" formatCells="0" formatColumns="0" formatRows="0" insertRows="0" deleteRows="0" sort="0" autoFilter="0"/>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D201">
       <formula1>"Chest,Front delts,Side delts,Rear delts,Triceps,Lats,Upper back,Traps,Biceps,Forearms,Quads,Hamstrings,Glutes,Adductors,Abductors,Calves,Abs,Obliques,Lower back,Neck"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" sqref="E2:E201">
       <formula1>"Chest,Front delts,Side delts,Rear delts,Triceps,Lats,Upper back,Traps,Biceps,Forearms,Quads,Hamstrings,Glutes,Adductors,Abductors,Calves,Abs,Obliques,Lower back,Neck"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Target max RPE" prompt="The hardest a set should feel: 1 to 10." errorTitle="Target max RPE" error="Enter a number from 1 to 10." sqref="I2:I201">
+      <formula1>1</formula1>
+      <formula2>10</formula2>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -2633,17 +2843,21 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rest is in SECONDS. 120 means two minutes.</t>
+          <t xml:space="preserve">Target max RPE is a CEILING from 1 to 10: the hardest a set should feel, 10 meaning nothing</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="0"/>
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">left. The app shows it grey during the session, and a set you leave unrated saves it as its rating.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do not rename, reorder or delete the header row - the import matches on those names.</t>
+          <t xml:space="preserve">Rest is in SECONDS. 120 means two minutes.</t>
         </is>
       </c>
     </row>
@@ -2651,185 +2865,195 @@
       <c r="A18" s="0"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Do not rename, reorder or delete the header row - the import matches on those names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Worked example</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Program        Exercise             Primary   Secondary          Sets Reps Weight Rest</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lower A        Leg Press midfoot    Quads     Glutes             3    10   50     90</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lower A        Lying Leg Curl       Hamstrings Calves            3    8    30     90</t>
+          <t xml:space="preserve">Program   Exercise            Primary     Secondary   Sets Reps Weight MaxRPE Rest</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lower A        Leg Extension        Quads                        3    12   40     60</t>
+          <t xml:space="preserve">Lower A   Leg Press midfoot   Quads       Glutes      3    10   50     8      90</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="0"/>
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lower A   Lying Leg Curl      Hamstrings  Calves      3    8    30     8      90</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lower A   Leg Extension       Quads                   3    12   40            60</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Muscle groups you can choose from</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chest</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Front delts</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Side delts</t>
+          <t xml:space="preserve">Chest</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rear delts</t>
+          <t xml:space="preserve">Front delts</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Triceps</t>
+          <t xml:space="preserve">Side delts</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lats</t>
+          <t xml:space="preserve">Rear delts</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upper back</t>
+          <t xml:space="preserve">Triceps</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Traps</t>
+          <t xml:space="preserve">Lats</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biceps</t>
+          <t xml:space="preserve">Upper back</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Forearms</t>
+          <t xml:space="preserve">Traps</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quads</t>
+          <t xml:space="preserve">Biceps</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hamstrings</t>
+          <t xml:space="preserve">Forearms</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glutes</t>
+          <t xml:space="preserve">Quads</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adductors</t>
+          <t xml:space="preserve">Hamstrings</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abductors</t>
+          <t xml:space="preserve">Glutes</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Calves</t>
+          <t xml:space="preserve">Adductors</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abs</t>
+          <t xml:space="preserve">Abductors</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obliques</t>
+          <t xml:space="preserve">Calves</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lower back</t>
+          <t xml:space="preserve">Abs</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obliques</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lower back</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Neck</t>
         </is>

</xml_diff>